<commit_message>
Merge the quads and quadMaps spec files into planes.md.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFB9AA1C-3CA1-D345-AC56-2A38218F533E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E134897-9DA5-BF41-A1B3-8F2999EF1816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
+    <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
   <sheets>
     <sheet name="Docs" sheetId="2" r:id="rId1"/>
@@ -885,7 +885,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -925,11 +925,32 @@
         <v>11</v>
       </c>
       <c r="E2" s="4">
-        <f t="shared" ref="E2" si="0">B2/D2</f>
+        <f t="shared" ref="E2:E3" si="0">B2/D2</f>
         <v>107.36363636363636</v>
       </c>
       <c r="F2">
         <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" s="6">
+        <v>46102</v>
+      </c>
+      <c r="B3">
+        <v>3330</v>
+      </c>
+      <c r="C3">
+        <v>74</v>
+      </c>
+      <c r="D3">
+        <v>18</v>
+      </c>
+      <c r="E3" s="4">
+        <f t="shared" si="0"/>
+        <v>185</v>
+      </c>
+      <c r="F3">
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Create the unitCells module.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E134897-9DA5-BF41-A1B3-8F2999EF1816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15BCD951-2349-E842-9C10-7E5C2DE263EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -885,7 +885,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -925,7 +925,7 @@
         <v>11</v>
       </c>
       <c r="E2" s="4">
-        <f t="shared" ref="E2:E3" si="0">B2/D2</f>
+        <f t="shared" ref="E2:E4" si="0">B2/D2</f>
         <v>107.36363636363636</v>
       </c>
       <c r="F2">
@@ -951,6 +951,27 @@
       </c>
       <c r="F3">
         <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" s="6">
+        <v>46104</v>
+      </c>
+      <c r="B4">
+        <v>3823</v>
+      </c>
+      <c r="C4">
+        <v>105</v>
+      </c>
+      <c r="D4">
+        <v>20</v>
+      </c>
+      <c r="E4" s="4">
+        <f t="shared" si="0"/>
+        <v>191.15</v>
+      </c>
+      <c r="F4">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Clean up the quads.md spec file.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D6834C2-D71A-0B46-A28F-DF4A0A08941A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F6D64C7-DF99-354A-B62E-192407631146}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -885,7 +885,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -925,7 +925,7 @@
         <v>11</v>
       </c>
       <c r="E2" s="4">
-        <f t="shared" ref="E2:E5" si="0">B2/D2</f>
+        <f t="shared" ref="E2:E6" si="0">B2/D2</f>
         <v>107.36363636363636</v>
       </c>
       <c r="F2">
@@ -993,6 +993,27 @@
       </c>
       <c r="F5">
         <v>69</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" s="6">
+        <v>46107</v>
+      </c>
+      <c r="B6">
+        <v>5553</v>
+      </c>
+      <c r="C6">
+        <v>166</v>
+      </c>
+      <c r="D6">
+        <v>24</v>
+      </c>
+      <c r="E6" s="4">
+        <f>B6/D6</f>
+        <v>231.375</v>
+      </c>
+      <c r="F6">
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AdvSq: first stable point.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5241F0AF-03A4-EF43-9C9F-700663E8EA47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{306E005A-E444-0B4F-A0F0-58C30F87C2ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -885,7 +885,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1037,6 +1037,27 @@
         <v>99</v>
       </c>
     </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" s="6">
+        <v>46111</v>
+      </c>
+      <c r="B8">
+        <v>5852</v>
+      </c>
+      <c r="C8">
+        <v>208</v>
+      </c>
+      <c r="D8">
+        <v>30</v>
+      </c>
+      <c r="E8" s="4">
+        <f>B8/D8</f>
+        <v>195.06666666666666</v>
+      </c>
+      <c r="F8">
+        <v>108</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Upgrade planes and quads with next and prev functions.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{306E005A-E444-0B4F-A0F0-58C30F87C2ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{593B7ED0-7F37-D847-B719-F68372F077A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -885,7 +885,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1058,6 +1058,27 @@
         <v>108</v>
       </c>
     </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" s="6">
+        <v>46112</v>
+      </c>
+      <c r="B9">
+        <v>5991</v>
+      </c>
+      <c r="C9">
+        <v>211</v>
+      </c>
+      <c r="D9">
+        <v>30</v>
+      </c>
+      <c r="E9" s="4">
+        <f>B9/D9</f>
+        <v>199.7</v>
+      </c>
+      <c r="F9">
+        <v>109</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
AdvSq: stable geometry + navigation + invariants
- Implement AdvSq constructors (quad, rayPair)
- Add perim assembly including k=0 degenerate case
- Implement next/prev quad and plane navigation
- Add structural accessors (E1, apex, E2, area, perims)
- Validate color invariants (bishop/duke)
- Add comprehensive regression tests (324 passing)

Establishes AdvSq as a stable geometric primitive.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{593B7ED0-7F37-D847-B719-F68372F077A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84B6EF3B-1756-9849-B7B8-CB7B605C0C11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -885,7 +885,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1079,6 +1079,27 @@
         <v>109</v>
       </c>
     </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" s="6">
+        <v>46113</v>
+      </c>
+      <c r="B10">
+        <v>6302</v>
+      </c>
+      <c r="C10">
+        <v>220</v>
+      </c>
+      <c r="D10">
+        <v>30</v>
+      </c>
+      <c r="E10" s="4">
+        <f>B10/D10</f>
+        <v>210.06666666666666</v>
+      </c>
+      <c r="F10">
+        <v>111</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Overhead and some qt3 cleanup.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84B6EF3B-1756-9849-B7B8-CB7B605C0C11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B268542-F59F-8D4B-ADBE-8F489E683124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -885,7 +885,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1100,6 +1100,27 @@
         <v>111</v>
       </c>
     </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" s="6">
+        <v>46114</v>
+      </c>
+      <c r="B11">
+        <v>6931</v>
+      </c>
+      <c r="C11">
+        <v>240</v>
+      </c>
+      <c r="D11">
+        <v>36</v>
+      </c>
+      <c r="E11" s="4">
+        <f>B11/D11</f>
+        <v>192.52777777777777</v>
+      </c>
+      <c r="F11">
+        <v>126</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
8x8x8 tiles, plumb dragable 2D control canvases, with names.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B268542-F59F-8D4B-ADBE-8F489E683124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{597ECA0D-FF45-4D4B-AD62-0673C3FD7585}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -885,7 +885,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1121,6 +1121,27 @@
         <v>126</v>
       </c>
     </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" s="6">
+        <v>46115</v>
+      </c>
+      <c r="B12">
+        <v>7178</v>
+      </c>
+      <c r="C12">
+        <v>246</v>
+      </c>
+      <c r="D12">
+        <v>39</v>
+      </c>
+      <c r="E12" s="4">
+        <f>B12/D12</f>
+        <v>184.05128205128204</v>
+      </c>
+      <c r="F12">
+        <v>124</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Nail down state for undo/redo.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{597ECA0D-FF45-4D4B-AD62-0673C3FD7585}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{176923AB-6C9E-CB41-B8DC-EA36A3E8922E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -885,7 +885,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1142,6 +1142,27 @@
         <v>124</v>
       </c>
     </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" s="6">
+        <v>46116</v>
+      </c>
+      <c r="B13">
+        <v>7673</v>
+      </c>
+      <c r="C13">
+        <v>259</v>
+      </c>
+      <c r="D13">
+        <v>40</v>
+      </c>
+      <c r="E13" s="4">
+        <f>B13/D13</f>
+        <v>191.82499999999999</v>
+      </c>
+      <c r="F13">
+        <v>129</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Start on model/state tests.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{176923AB-6C9E-CB41-B8DC-EA36A3E8922E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EBEC222-D537-5E4D-A050-9FDA6F690353}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -885,7 +885,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1163,6 +1163,27 @@
         <v>129</v>
       </c>
     </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" s="6">
+        <v>46117</v>
+      </c>
+      <c r="B14">
+        <v>7739</v>
+      </c>
+      <c r="C14">
+        <v>263</v>
+      </c>
+      <c r="D14">
+        <v>41</v>
+      </c>
+      <c r="E14" s="4">
+        <f>B14/D14</f>
+        <v>188.7560975609756</v>
+      </c>
+      <c r="F14">
+        <v>132</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
State module for undo/redoable state.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EBEC222-D537-5E4D-A050-9FDA6F690353}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C6CCCE6-093E-8546-AD00-DA1B6795736D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -885,7 +885,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -925,7 +925,7 @@
         <v>11</v>
       </c>
       <c r="E2" s="4">
-        <f t="shared" ref="E2:E6" si="0">B2/D2</f>
+        <f t="shared" ref="E2:E5" si="0">B2/D2</f>
         <v>107.36363636363636</v>
       </c>
       <c r="F2">
@@ -1009,7 +1009,7 @@
         <v>24</v>
       </c>
       <c r="E6" s="4">
-        <f>B6/D6</f>
+        <f t="shared" ref="E6:E15" si="1">B6/D6</f>
         <v>231.375</v>
       </c>
       <c r="F6">
@@ -1030,7 +1030,7 @@
         <v>26</v>
       </c>
       <c r="E7" s="4">
-        <f>B7/D7</f>
+        <f t="shared" si="1"/>
         <v>169.26923076923077</v>
       </c>
       <c r="F7">
@@ -1051,7 +1051,7 @@
         <v>30</v>
       </c>
       <c r="E8" s="4">
-        <f>B8/D8</f>
+        <f t="shared" si="1"/>
         <v>195.06666666666666</v>
       </c>
       <c r="F8">
@@ -1072,7 +1072,7 @@
         <v>30</v>
       </c>
       <c r="E9" s="4">
-        <f>B9/D9</f>
+        <f t="shared" si="1"/>
         <v>199.7</v>
       </c>
       <c r="F9">
@@ -1093,7 +1093,7 @@
         <v>30</v>
       </c>
       <c r="E10" s="4">
-        <f>B10/D10</f>
+        <f t="shared" si="1"/>
         <v>210.06666666666666</v>
       </c>
       <c r="F10">
@@ -1114,7 +1114,7 @@
         <v>36</v>
       </c>
       <c r="E11" s="4">
-        <f>B11/D11</f>
+        <f t="shared" si="1"/>
         <v>192.52777777777777</v>
       </c>
       <c r="F11">
@@ -1135,7 +1135,7 @@
         <v>39</v>
       </c>
       <c r="E12" s="4">
-        <f>B12/D12</f>
+        <f t="shared" si="1"/>
         <v>184.05128205128204</v>
       </c>
       <c r="F12">
@@ -1156,7 +1156,7 @@
         <v>40</v>
       </c>
       <c r="E13" s="4">
-        <f>B13/D13</f>
+        <f t="shared" si="1"/>
         <v>191.82499999999999</v>
       </c>
       <c r="F13">
@@ -1177,11 +1177,32 @@
         <v>41</v>
       </c>
       <c r="E14" s="4">
-        <f>B14/D14</f>
+        <f t="shared" si="1"/>
         <v>188.7560975609756</v>
       </c>
       <c r="F14">
         <v>132</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" s="6">
+        <v>46118</v>
+      </c>
+      <c r="B15">
+        <v>8183</v>
+      </c>
+      <c r="C15">
+        <v>275</v>
+      </c>
+      <c r="D15">
+        <v>42</v>
+      </c>
+      <c r="E15" s="4">
+        <f t="shared" si="1"/>
+        <v>194.83333333333334</v>
+      </c>
+      <c r="F15">
+        <v>139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update project spreadsheet & git-notes.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{269D92A8-A336-684C-BBA4-CD94E84F0B21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB53C78C-F669-954F-BFC2-34323FCE6A6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -885,7 +885,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1009,7 +1009,7 @@
         <v>24</v>
       </c>
       <c r="E6" s="4">
-        <f t="shared" ref="E6:E16" si="1">B6/D6</f>
+        <f t="shared" ref="E6:E18" si="1">B6/D6</f>
         <v>231.375</v>
       </c>
       <c r="F6">
@@ -1224,6 +1224,33 @@
       </c>
       <c r="F16">
         <v>153</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" s="6">
+        <v>46120</v>
+      </c>
+      <c r="E17" s="4"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" s="6">
+        <v>46121</v>
+      </c>
+      <c r="B18">
+        <v>9559</v>
+      </c>
+      <c r="C18">
+        <v>359</v>
+      </c>
+      <c r="D18">
+        <v>46</v>
+      </c>
+      <c r="E18" s="4">
+        <f t="shared" si="1"/>
+        <v>207.80434782608697</v>
+      </c>
+      <c r="F18">
+        <v>171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add 3rd panel, continue refining panel arch.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1864227F-DC68-A54C-9BED-04D890A7BC01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{854E01C4-7B5C-964F-9333-43EF17B987CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -885,7 +885,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1274,6 +1274,11 @@
         <v>180</v>
       </c>
     </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A20" s="6">
+        <v>46123</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 5th panel: setup, tray, game, gambit, camera.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{854E01C4-7B5C-964F-9333-43EF17B987CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD048C18-1E82-A64D-8404-9B5CD29F1B2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -1009,7 +1009,7 @@
         <v>24</v>
       </c>
       <c r="E6" s="4">
-        <f t="shared" ref="E6:E19" si="1">B6/D6</f>
+        <f t="shared" ref="E6:E20" si="1">B6/D6</f>
         <v>231.375</v>
       </c>
       <c r="F6">
@@ -1277,6 +1277,22 @@
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="6">
         <v>46123</v>
+      </c>
+      <c r="B20">
+        <v>10382</v>
+      </c>
+      <c r="C20">
+        <v>419</v>
+      </c>
+      <c r="D20">
+        <v>49</v>
+      </c>
+      <c r="E20" s="4">
+        <f t="shared" si="1"/>
+        <v>211.87755102040816</v>
+      </c>
+      <c r="F20">
+        <v>184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Make camera POV radio buttons active elements.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD048C18-1E82-A64D-8404-9B5CD29F1B2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85B557A1-B303-B041-8EF6-5C720E8198E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -177,7 +177,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -192,6 +192,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -885,17 +889,18 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
+    <col min="2" max="2" width="10.83203125" style="9"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -915,7 +920,7 @@
       <c r="A2" s="6">
         <v>46100</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="9">
         <v>1181</v>
       </c>
       <c r="C2">
@@ -936,7 +941,7 @@
       <c r="A3" s="6">
         <v>46102</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="9">
         <v>3330</v>
       </c>
       <c r="C3">
@@ -957,7 +962,7 @@
       <c r="A4" s="6">
         <v>46104</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="9">
         <v>3823</v>
       </c>
       <c r="C4">
@@ -978,7 +983,7 @@
       <c r="A5" s="6">
         <v>46105</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="9">
         <v>3951</v>
       </c>
       <c r="C5">
@@ -999,7 +1004,7 @@
       <c r="A6" s="6">
         <v>46107</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="9">
         <v>5553</v>
       </c>
       <c r="C6">
@@ -1020,7 +1025,7 @@
       <c r="A7" s="6">
         <v>46108</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="9">
         <v>4401</v>
       </c>
       <c r="C7">
@@ -1041,7 +1046,7 @@
       <c r="A8" s="6">
         <v>46111</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="9">
         <v>5852</v>
       </c>
       <c r="C8">
@@ -1062,7 +1067,7 @@
       <c r="A9" s="6">
         <v>46112</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="9">
         <v>5991</v>
       </c>
       <c r="C9">
@@ -1083,7 +1088,7 @@
       <c r="A10" s="6">
         <v>46113</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="9">
         <v>6302</v>
       </c>
       <c r="C10">
@@ -1104,7 +1109,7 @@
       <c r="A11" s="6">
         <v>46114</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="9">
         <v>6931</v>
       </c>
       <c r="C11">
@@ -1125,7 +1130,7 @@
       <c r="A12" s="6">
         <v>46115</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="9">
         <v>7178</v>
       </c>
       <c r="C12">
@@ -1146,7 +1151,7 @@
       <c r="A13" s="6">
         <v>46116</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="9">
         <v>7673</v>
       </c>
       <c r="C13">
@@ -1167,7 +1172,7 @@
       <c r="A14" s="6">
         <v>46117</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="9">
         <v>7739</v>
       </c>
       <c r="C14">
@@ -1188,7 +1193,7 @@
       <c r="A15" s="6">
         <v>46118</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="9">
         <v>8183</v>
       </c>
       <c r="C15">
@@ -1209,7 +1214,7 @@
       <c r="A16" s="6">
         <v>46119</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="9">
         <v>8610</v>
       </c>
       <c r="C16">
@@ -1236,7 +1241,7 @@
       <c r="A18" s="6">
         <v>46121</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="9">
         <v>9559</v>
       </c>
       <c r="C18">
@@ -1257,7 +1262,7 @@
       <c r="A19" s="6">
         <v>46122</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="9">
         <v>10064</v>
       </c>
       <c r="C19">
@@ -1278,7 +1283,7 @@
       <c r="A20" s="6">
         <v>46123</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="9">
         <v>10382</v>
       </c>
       <c r="C20">
@@ -1293,6 +1298,11 @@
       </c>
       <c r="F20">
         <v>184</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A21" s="6">
+        <v>46124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add 7th panel: move listing.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85B557A1-B303-B041-8EF6-5C720E8198E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92831BFD-33B6-B74E-A642-04076BB631A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -1014,7 +1014,7 @@
         <v>24</v>
       </c>
       <c r="E6" s="4">
-        <f t="shared" ref="E6:E20" si="1">B6/D6</f>
+        <f t="shared" ref="E6:E21" si="1">B6/D6</f>
         <v>231.375</v>
       </c>
       <c r="F6">
@@ -1303,6 +1303,22 @@
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="6">
         <v>46124</v>
+      </c>
+      <c r="B21" s="9">
+        <v>10511</v>
+      </c>
+      <c r="C21">
+        <v>429</v>
+      </c>
+      <c r="D21">
+        <v>49</v>
+      </c>
+      <c r="E21" s="4">
+        <f t="shared" si="1"/>
+        <v>214.51020408163265</v>
+      </c>
+      <c r="F21">
+        <v>185</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Prep for post merge.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92831BFD-33B6-B74E-A642-04076BB631A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{614DECE6-03ED-4D46-A44F-0C03C76C2652}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -1014,7 +1014,7 @@
         <v>24</v>
       </c>
       <c r="E6" s="4">
-        <f t="shared" ref="E6:E21" si="1">B6/D6</f>
+        <f t="shared" ref="E6:E34" si="1">B6/D6</f>
         <v>231.375</v>
       </c>
       <c r="F6">
@@ -1305,17 +1305,17 @@
         <v>46124</v>
       </c>
       <c r="B21" s="9">
-        <v>10511</v>
+        <v>10411</v>
       </c>
       <c r="C21">
-        <v>429</v>
+        <v>425</v>
       </c>
       <c r="D21">
         <v>49</v>
       </c>
       <c r="E21" s="4">
-        <f t="shared" si="1"/>
-        <v>214.51020408163265</v>
+        <f t="shared" ref="E21" si="2">B21/D21</f>
+        <v>212.46938775510205</v>
       </c>
       <c r="F21">
         <v>185</v>

</xml_diff>

<commit_message>
Clean up DOM panel code.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{614DECE6-03ED-4D46-A44F-0C03C76C2652}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{386C3E68-FD6A-304D-AB1E-02168401C27D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -889,7 +889,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1321,6 +1321,14 @@
         <v>185</v>
       </c>
     </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" s="6">
+        <v>46125</v>
+      </c>
+      <c r="B22" s="9">
+        <v>10334</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
First pass on logarithmic undo (current state off-by-one error).
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{386C3E68-FD6A-304D-AB1E-02168401C27D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{569F1763-B09F-6947-B228-1817876F953F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -1314,7 +1314,7 @@
         <v>49</v>
       </c>
       <c r="E21" s="4">
-        <f t="shared" ref="E21" si="2">B21/D21</f>
+        <f t="shared" ref="E21:E22" si="2">B21/D21</f>
         <v>212.46938775510205</v>
       </c>
       <c r="F21">
@@ -1326,7 +1326,20 @@
         <v>46125</v>
       </c>
       <c r="B22" s="9">
-        <v>10334</v>
+        <v>10383</v>
+      </c>
+      <c r="C22">
+        <v>423</v>
+      </c>
+      <c r="D22">
+        <v>49</v>
+      </c>
+      <c r="E22" s="4">
+        <f t="shared" si="2"/>
+        <v>211.89795918367346</v>
+      </c>
+      <c r="F22">
+        <v>188</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix undo/redo/rerun to deal with setup edge case (no board).
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{569F1763-B09F-6947-B228-1817876F953F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97018C4C-061D-C04F-8037-64C507C45C76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -889,7 +889,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1314,7 +1314,7 @@
         <v>49</v>
       </c>
       <c r="E21" s="4">
-        <f t="shared" ref="E21:E22" si="2">B21/D21</f>
+        <f t="shared" ref="E21:E23" si="2">B21/D21</f>
         <v>212.46938775510205</v>
       </c>
       <c r="F21">
@@ -1340,6 +1340,27 @@
       </c>
       <c r="F22">
         <v>188</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A23" s="6">
+        <v>46126</v>
+      </c>
+      <c r="B23" s="9">
+        <v>10646</v>
+      </c>
+      <c r="C23">
+        <v>435</v>
+      </c>
+      <c r="D23">
+        <v>50</v>
+      </c>
+      <c r="E23" s="4">
+        <f t="shared" si="2"/>
+        <v>212.92</v>
+      </c>
+      <c r="F23">
+        <v>191</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Undo/redo working, rerun not zeroing downstream elements.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97018C4C-061D-C04F-8037-64C507C45C76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{103D7CCF-E304-E04D-B191-D7C7C6A587B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -889,7 +889,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1314,7 +1314,7 @@
         <v>49</v>
       </c>
       <c r="E21" s="4">
-        <f t="shared" ref="E21:E23" si="2">B21/D21</f>
+        <f t="shared" ref="E21:E24" si="2">B21/D21</f>
         <v>212.46938775510205</v>
       </c>
       <c r="F21">
@@ -1361,6 +1361,27 @@
       </c>
       <c r="F23">
         <v>191</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A24" s="6">
+        <v>46127</v>
+      </c>
+      <c r="B24" s="9">
+        <v>10976</v>
+      </c>
+      <c r="C24">
+        <v>453</v>
+      </c>
+      <c r="D24">
+        <v>51</v>
+      </c>
+      <c r="E24" s="4">
+        <f t="shared" si="2"/>
+        <v>215.21568627450981</v>
+      </c>
+      <c r="F24">
+        <v>199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Advsq panel Remove feature.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFBED4B6-EE66-F649-8A66-755BD4695B9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B43CE5EA-8D61-F04A-95DC-CBB59305FD0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -889,7 +889,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1389,20 +1389,25 @@
         <v>46128</v>
       </c>
       <c r="B25" s="9">
-        <v>11110</v>
+        <v>11074</v>
       </c>
       <c r="C25">
         <v>453</v>
       </c>
       <c r="D25">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E25" s="4">
         <f t="shared" si="2"/>
-        <v>217.84313725490196</v>
+        <v>221.48</v>
       </c>
       <c r="F25">
         <v>200</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A26" s="6">
+        <v>46129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
dd stride tile to use dst decorator.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BF26CF7-4C8C-7E41-B34C-7A22CF7A1E92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0832324-C854-AA4E-8748-984F09D410DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -889,7 +889,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1314,7 +1314,7 @@
         <v>49</v>
       </c>
       <c r="E21" s="4">
-        <f t="shared" ref="E21:E26" si="2">B21/D21</f>
+        <f t="shared" ref="E21:E27" si="2">B21/D21</f>
         <v>212.46938775510205</v>
       </c>
       <c r="F21">
@@ -1424,6 +1424,27 @@
       </c>
       <c r="F26">
         <v>207</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A27" s="6">
+        <v>46130</v>
+      </c>
+      <c r="B27" s="9">
+        <v>11368</v>
+      </c>
+      <c r="C27">
+        <v>465</v>
+      </c>
+      <c r="D27">
+        <v>50</v>
+      </c>
+      <c r="E27" s="4">
+        <f t="shared" si="2"/>
+        <v>227.36</v>
+      </c>
+      <c r="F27">
+        <v>204</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Move thirds from edge to face quads.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0832324-C854-AA4E-8748-984F09D410DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B26538F1-5874-2B40-A510-FFF42E63DBE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -889,7 +889,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1014,7 +1014,7 @@
         <v>24</v>
       </c>
       <c r="E6" s="4">
-        <f t="shared" ref="E6:E34" si="1">B6/D6</f>
+        <f t="shared" ref="E6:E19" si="1">B6/D6</f>
         <v>231.375</v>
       </c>
       <c r="F6">
@@ -1233,218 +1233,238 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="6">
-        <v>46120</v>
-      </c>
-      <c r="E17" s="4"/>
+        <v>46121</v>
+      </c>
+      <c r="B17" s="9">
+        <v>9559</v>
+      </c>
+      <c r="C17">
+        <v>359</v>
+      </c>
+      <c r="D17">
+        <v>46</v>
+      </c>
+      <c r="E17" s="4">
+        <f t="shared" si="1"/>
+        <v>207.80434782608697</v>
+      </c>
+      <c r="F17">
+        <v>171</v>
+      </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="6">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B18" s="9">
-        <v>9559</v>
+        <v>10064</v>
       </c>
       <c r="C18">
-        <v>359</v>
+        <v>389</v>
       </c>
       <c r="D18">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E18" s="4">
         <f t="shared" si="1"/>
-        <v>207.80434782608697</v>
+        <v>205.38775510204081</v>
       </c>
       <c r="F18">
-        <v>171</v>
+        <v>180</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="6">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B19" s="9">
-        <v>10064</v>
+        <v>10382</v>
       </c>
       <c r="C19">
-        <v>389</v>
+        <v>419</v>
       </c>
       <c r="D19">
         <v>49</v>
       </c>
       <c r="E19" s="4">
         <f t="shared" si="1"/>
-        <v>205.38775510204081</v>
+        <v>211.87755102040816</v>
       </c>
       <c r="F19">
-        <v>180</v>
+        <v>184</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="6">
-        <v>46123</v>
+        <v>46124</v>
       </c>
       <c r="B20" s="9">
-        <v>10382</v>
+        <v>10411</v>
       </c>
       <c r="C20">
-        <v>419</v>
+        <v>425</v>
       </c>
       <c r="D20">
         <v>49</v>
       </c>
       <c r="E20" s="4">
-        <f t="shared" si="1"/>
-        <v>211.87755102040816</v>
+        <f t="shared" ref="E20:E27" si="2">B20/D20</f>
+        <v>212.46938775510205</v>
       </c>
       <c r="F20">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="6">
-        <v>46124</v>
+        <v>46125</v>
       </c>
       <c r="B21" s="9">
-        <v>10411</v>
+        <v>10383</v>
       </c>
       <c r="C21">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="D21">
         <v>49</v>
       </c>
       <c r="E21" s="4">
-        <f t="shared" ref="E21:E27" si="2">B21/D21</f>
-        <v>212.46938775510205</v>
+        <f t="shared" si="2"/>
+        <v>211.89795918367346</v>
       </c>
       <c r="F21">
-        <v>185</v>
+        <v>188</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="6">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B22" s="9">
-        <v>10383</v>
+        <v>10646</v>
       </c>
       <c r="C22">
-        <v>423</v>
+        <v>435</v>
       </c>
       <c r="D22">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E22" s="4">
         <f t="shared" si="2"/>
-        <v>211.89795918367346</v>
+        <v>212.92</v>
       </c>
       <c r="F22">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="6">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B23" s="9">
-        <v>10646</v>
+        <v>10976</v>
       </c>
       <c r="C23">
-        <v>435</v>
+        <v>453</v>
       </c>
       <c r="D23">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E23" s="4">
         <f t="shared" si="2"/>
-        <v>212.92</v>
+        <v>215.21568627450981</v>
       </c>
       <c r="F23">
-        <v>191</v>
+        <v>199</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="6">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B24" s="9">
-        <v>10976</v>
+        <v>11074</v>
       </c>
       <c r="C24">
         <v>453</v>
       </c>
       <c r="D24">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E24" s="4">
         <f t="shared" si="2"/>
-        <v>215.21568627450981</v>
+        <v>221.48</v>
       </c>
       <c r="F24">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="6">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B25" s="9">
-        <v>11074</v>
+        <v>11386</v>
       </c>
       <c r="C25">
-        <v>453</v>
+        <v>467</v>
       </c>
       <c r="D25">
         <v>50</v>
       </c>
       <c r="E25" s="4">
         <f t="shared" si="2"/>
-        <v>221.48</v>
+        <v>227.72</v>
       </c>
       <c r="F25">
-        <v>200</v>
+        <v>207</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="6">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B26" s="9">
-        <v>11386</v>
+        <v>11368</v>
       </c>
       <c r="C26">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="D26">
         <v>50</v>
       </c>
       <c r="E26" s="4">
         <f t="shared" si="2"/>
-        <v>227.72</v>
+        <v>227.36</v>
       </c>
       <c r="F26">
-        <v>207</v>
+        <v>204</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="6">
-        <v>46130</v>
+        <v>46131</v>
       </c>
       <c r="B27" s="9">
-        <v>11368</v>
+        <v>11424</v>
       </c>
       <c r="C27">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="D27">
         <v>50</v>
       </c>
       <c r="E27" s="4">
         <f t="shared" si="2"/>
-        <v>227.36</v>
+        <v>228.48</v>
       </c>
       <c r="F27">
         <v>204</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A28" s="6">
+        <v>46132</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Move advsq control into its own dir.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B26538F1-5874-2B40-A510-FFF42E63DBE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3516BBF-4E2D-6A4A-A602-EFDF462BBE12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -1308,7 +1308,7 @@
         <v>49</v>
       </c>
       <c r="E20" s="4">
-        <f t="shared" ref="E20:E27" si="2">B20/D20</f>
+        <f t="shared" ref="E20:E28" si="2">B20/D20</f>
         <v>212.46938775510205</v>
       </c>
       <c r="F20">
@@ -1465,6 +1465,22 @@
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="6">
         <v>46132</v>
+      </c>
+      <c r="B28" s="9">
+        <v>11771</v>
+      </c>
+      <c r="C28">
+        <v>483</v>
+      </c>
+      <c r="D28">
+        <v>51</v>
+      </c>
+      <c r="E28" s="4">
+        <f t="shared" si="2"/>
+        <v>230.80392156862746</v>
+      </c>
+      <c r="F28">
+        <v>214</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add grow and shrink to advsq panel, better intuition and MVC compliance.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3516BBF-4E2D-6A4A-A602-EFDF462BBE12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6AD0A84-489A-D84C-828A-E366151CFD03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -889,7 +889,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1308,7 +1308,7 @@
         <v>49</v>
       </c>
       <c r="E20" s="4">
-        <f t="shared" ref="E20:E28" si="2">B20/D20</f>
+        <f t="shared" ref="E20:E29" si="2">B20/D20</f>
         <v>212.46938775510205</v>
       </c>
       <c r="F20">
@@ -1481,6 +1481,27 @@
       </c>
       <c r="F28">
         <v>214</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A29" s="6">
+        <v>46133</v>
+      </c>
+      <c r="B29" s="9">
+        <v>11439</v>
+      </c>
+      <c r="C29">
+        <v>470</v>
+      </c>
+      <c r="D29">
+        <v>51</v>
+      </c>
+      <c r="E29" s="4">
+        <f t="shared" si="2"/>
+        <v>224.29411764705881</v>
+      </c>
+      <c r="F29">
+        <v>215</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Attempt max stride limit.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6AD0A84-489A-D84C-828A-E366151CFD03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F4B2FFB-E883-5544-B706-D1F08CA2AE78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -889,7 +889,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1504,6 +1504,11 @@
         <v>215</v>
       </c>
     </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A30" s="6">
+        <v>46134</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add state level undo/redo.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D93354C2-CF55-4D4E-A944-A8338767FA85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{733BCAEB-2C24-CE4A-93DF-0570BFBF9469}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -1509,20 +1509,20 @@
         <v>46134</v>
       </c>
       <c r="B30" s="9">
-        <v>12055</v>
+        <v>12218</v>
       </c>
       <c r="C30">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="D30">
         <v>53</v>
       </c>
       <c r="E30" s="4">
         <f t="shared" si="2"/>
-        <v>227.45283018867926</v>
+        <v>230.52830188679246</v>
       </c>
       <c r="F30">
-        <v>229</v>
+        <v>233</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor advsqs to use state undo.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{733BCAEB-2C24-CE4A-93DF-0570BFBF9469}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E26D72B5-802D-7C4D-8360-5A768832D307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -889,7 +889,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1525,6 +1525,11 @@
         <v>233</v>
       </c>
     </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A31" s="6">
+        <v>46135</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Delete undo system at control layer.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E26D72B5-802D-7C4D-8360-5A768832D307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F02B577-64D2-1540-AAD9-60F38F9E8F65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-21000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -1308,7 +1308,7 @@
         <v>49</v>
       </c>
       <c r="E20" s="4">
-        <f t="shared" ref="E20:E30" si="2">B20/D20</f>
+        <f t="shared" ref="E20:E31" si="2">B20/D20</f>
         <v>212.46938775510205</v>
       </c>
       <c r="F20">
@@ -1528,6 +1528,22 @@
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="6">
         <v>46135</v>
+      </c>
+      <c r="B31" s="9">
+        <v>11749</v>
+      </c>
+      <c r="C31">
+        <v>481</v>
+      </c>
+      <c r="D31">
+        <v>53</v>
+      </c>
+      <c r="E31" s="4">
+        <f t="shared" si="2"/>
+        <v>221.67924528301887</v>
+      </c>
+      <c r="F31">
+        <v>220</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor to one wirePanel function.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1B68972-6803-B242-B146-2D3C27F1B8C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C68F5E1F-A4D7-6843-8967-E24C611452E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -893,7 +893,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1315,7 +1315,7 @@
         <v>49</v>
       </c>
       <c r="E20" s="4">
-        <f t="shared" ref="E20:E35" si="2">B20/D20</f>
+        <f t="shared" ref="E20:E36" si="2">B20/D20</f>
         <v>212.46938775510205</v>
       </c>
       <c r="F20">
@@ -1650,6 +1650,27 @@
       </c>
       <c r="G35">
         <v>30</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B36" s="9">
+        <v>12713</v>
+      </c>
+      <c r="C36">
+        <v>514</v>
+      </c>
+      <c r="D36">
+        <v>56</v>
+      </c>
+      <c r="E36" s="4">
+        <f t="shared" si="2"/>
+        <v>227.01785714285714</v>
+      </c>
+      <c r="F36">
+        <v>234</v>
+      </c>
+      <c r="G36">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Order panels in controller.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C68F5E1F-A4D7-6843-8967-E24C611452E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75803C39-EC7B-5F47-BF3A-5E25C933311D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -1654,23 +1654,23 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B36" s="9">
-        <v>12713</v>
+        <v>12572</v>
       </c>
       <c r="C36">
-        <v>514</v>
+        <v>509</v>
       </c>
       <c r="D36">
         <v>56</v>
       </c>
       <c r="E36" s="4">
         <f t="shared" si="2"/>
-        <v>227.01785714285714</v>
+        <v>224.5</v>
       </c>
       <c r="F36">
         <v>234</v>
       </c>
       <c r="G36">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Smooth jitter plus double click reverse.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1A282B6-BC63-9240-B364-AF0DAA2F34CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBDCB998-D89D-9341-9D1D-59E1E82BB127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -893,7 +893,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1652,6 +1652,11 @@
         <v>27</v>
       </c>
     </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A36" s="6">
+        <v>46140</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Clues & disable unimplemented panel features.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CD5C9EC-99FD-3F48-9AF3-CB42AD2FC129}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7021883D-6C6F-6247-B75C-50F2B17351DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -1681,23 +1681,23 @@
         <v>46141</v>
       </c>
       <c r="B37" s="9">
-        <v>12354</v>
+        <v>12567</v>
       </c>
       <c r="C37">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="D37">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="E37" s="4">
         <f t="shared" si="3"/>
-        <v>199.25806451612902</v>
+        <v>187.56716417910448</v>
       </c>
       <c r="F37">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="G37">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Replace bufferCount with bufferIndex.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88E83264-5EA7-1E49-9703-12D2DC3DE257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C24B02A-1D84-8E4D-9E48-6E04991B42AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -908,7 +908,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1763,6 +1763,11 @@
         <v>43</v>
       </c>
     </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A40" s="6">
+        <v>46144</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Time symmetric idiom for moves.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C24B02A-1D84-8E4D-9E48-6E04991B42AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6127E35-650C-AA4C-AF26-62C23CF37182}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -1767,6 +1767,9 @@
       <c r="A40" s="6">
         <v>46144</v>
       </c>
+      <c r="G40">
+        <v>48</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Expand MVC idiom for moves.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6127E35-650C-AA4C-AF26-62C23CF37182}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{716952D4-E9B4-654B-AD66-79F2016900A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -1681,7 +1681,7 @@
         <v>60</v>
       </c>
       <c r="E36" s="4">
-        <f t="shared" ref="E36:E39" si="3">B36/D36</f>
+        <f t="shared" ref="E36:E40" si="3">B36/D36</f>
         <v>201.96666666666667</v>
       </c>
       <c r="F36">
@@ -1767,8 +1767,24 @@
       <c r="A40" s="6">
         <v>46144</v>
       </c>
+      <c r="B40" s="9">
+        <v>13033</v>
+      </c>
+      <c r="C40">
+        <v>599</v>
+      </c>
+      <c r="D40">
+        <v>63</v>
+      </c>
+      <c r="E40" s="4">
+        <f t="shared" si="3"/>
+        <v>206.87301587301587</v>
+      </c>
+      <c r="F40">
+        <v>279</v>
+      </c>
       <c r="G40">
-        <v>48</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UI standardization model layer.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{716952D4-E9B4-654B-AD66-79F2016900A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8321D990-3C3A-DC45-B534-F577BF77B893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -1768,23 +1768,23 @@
         <v>46144</v>
       </c>
       <c r="B40" s="9">
-        <v>13033</v>
+        <v>13351</v>
       </c>
       <c r="C40">
-        <v>599</v>
+        <v>651</v>
       </c>
       <c r="D40">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E40" s="4">
         <f t="shared" si="3"/>
-        <v>206.87301587301587</v>
+        <v>208.609375</v>
       </c>
       <c r="F40">
-        <v>279</v>
+        <v>327</v>
       </c>
       <c r="G40">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Draft common UI functions for model layer.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8321D990-3C3A-DC45-B534-F577BF77B893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75925B45-42A8-D243-81AC-1E6DD2443598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -908,7 +908,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1787,6 +1787,11 @@
         <v>53</v>
       </c>
     </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A41" s="6">
+        <v>46145</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Complete state UI functions.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75925B45-42A8-D243-81AC-1E6DD2443598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{241C7B17-E31F-834C-B915-872014EE068A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -1681,7 +1681,7 @@
         <v>60</v>
       </c>
       <c r="E36" s="4">
-        <f t="shared" ref="E36:E40" si="3">B36/D36</f>
+        <f t="shared" ref="E36:E41" si="3">B36/D36</f>
         <v>201.96666666666667</v>
       </c>
       <c r="F36">
@@ -1790,6 +1790,25 @@
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" s="6">
         <v>46145</v>
+      </c>
+      <c r="B41" s="9">
+        <v>13767</v>
+      </c>
+      <c r="C41">
+        <v>657</v>
+      </c>
+      <c r="D41">
+        <v>64</v>
+      </c>
+      <c r="E41" s="4">
+        <f t="shared" si="3"/>
+        <v>215.109375</v>
+      </c>
+      <c r="F41">
+        <v>332</v>
+      </c>
+      <c r="G41">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add setup dir in view layer.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{241C7B17-E31F-834C-B915-872014EE068A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A608D06-CB37-5D48-A204-120E8A2037C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -1792,20 +1792,20 @@
         <v>46145</v>
       </c>
       <c r="B41" s="9">
-        <v>13767</v>
+        <v>13811</v>
       </c>
       <c r="C41">
-        <v>657</v>
+        <v>660</v>
       </c>
       <c r="D41">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E41" s="4">
         <f t="shared" si="3"/>
-        <v>215.109375</v>
+        <v>212.47692307692307</v>
       </c>
       <c r="F41">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="G41">
         <v>57</v>

</xml_diff>

<commit_message>
Debug undo/redo and refresh panel.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A608D06-CB37-5D48-A204-120E8A2037C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3FE0038-40D9-1846-B4C5-3704BE984A82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -908,7 +908,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1330,7 +1330,7 @@
         <v>49</v>
       </c>
       <c r="E20" s="4">
-        <f t="shared" ref="E20:E37" si="2">B20/D20</f>
+        <f t="shared" ref="E20:E35" si="2">B20/D20</f>
         <v>212.46938775510205</v>
       </c>
       <c r="F20">
@@ -1681,7 +1681,7 @@
         <v>60</v>
       </c>
       <c r="E36" s="4">
-        <f t="shared" ref="E36:E41" si="3">B36/D36</f>
+        <f t="shared" ref="E36:E42" si="3">B36/D36</f>
         <v>201.96666666666667</v>
       </c>
       <c r="F36">
@@ -1809,6 +1809,35 @@
       </c>
       <c r="G41">
         <v>57</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A42" s="6">
+        <v>46146</v>
+      </c>
+      <c r="B42" s="9">
+        <v>14753</v>
+      </c>
+      <c r="C42">
+        <v>689</v>
+      </c>
+      <c r="D42">
+        <v>68</v>
+      </c>
+      <c r="E42" s="4">
+        <f t="shared" si="3"/>
+        <v>216.95588235294119</v>
+      </c>
+      <c r="F42">
+        <v>352</v>
+      </c>
+      <c r="G42">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A43" s="6">
+        <v>46147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Apply pipeline canon to advsqs.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7D9471B-EC82-A24F-9169-FAFC3955A43F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89925289-300F-F040-85D7-2368784336F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -1840,23 +1840,23 @@
         <v>46147</v>
       </c>
       <c r="B43" s="9">
-        <v>14899</v>
+        <v>15018</v>
       </c>
       <c r="C43">
-        <v>696</v>
+        <v>699</v>
       </c>
       <c r="D43">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E43" s="4">
         <f t="shared" si="3"/>
-        <v>219.10294117647058</v>
+        <v>217.65217391304347</v>
       </c>
       <c r="F43">
         <v>358</v>
       </c>
       <c r="G43">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix redo on load.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77768869-6BE6-4D45-AA55-1FB91D3FCF9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12C85DD6-784F-1D46-B6AF-AE83613199DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -908,7 +908,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1907,6 +1907,11 @@
         <v>57</v>
       </c>
     </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A46" s="6">
+        <v>46149</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Re-arch view into panels.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A39537D-BFF4-F044-879B-50A433A300C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3BDC277-C34C-CA45-807D-F891D6C000BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -1873,7 +1873,7 @@
         <v>69</v>
       </c>
       <c r="E44" s="4">
-        <f t="shared" ref="E44:E46" si="4">B44/D44</f>
+        <f t="shared" ref="E44:E47" si="4">B44/D44</f>
         <v>217.65217391304347</v>
       </c>
       <c r="F44">
@@ -1934,6 +1934,25 @@
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" s="6">
         <v>46151</v>
+      </c>
+      <c r="B47" s="9">
+        <v>15320</v>
+      </c>
+      <c r="C47">
+        <v>708</v>
+      </c>
+      <c r="D47">
+        <v>70</v>
+      </c>
+      <c r="E47" s="4">
+        <f t="shared" si="4"/>
+        <v>218.85714285714286</v>
+      </c>
+      <c r="F47">
+        <v>365</v>
+      </c>
+      <c r="G47">
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Gambit specs and json files.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{859C0EB5-BE14-3542-8E07-9BA23200459E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B256BE3C-9B2A-DA47-9723-11F6695D63BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -908,7 +908,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1873,7 +1873,7 @@
         <v>69</v>
       </c>
       <c r="E44" s="4">
-        <f t="shared" ref="E44:E48" si="4">B44/D44</f>
+        <f t="shared" ref="E44:E49" si="4">B44/D44</f>
         <v>217.65217391304347</v>
       </c>
       <c r="F44">
@@ -1977,6 +1977,30 @@
       </c>
       <c r="G48">
         <v>58</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A49" s="6">
+        <v>46153</v>
+      </c>
+      <c r="B49" s="9">
+        <v>15862</v>
+      </c>
+      <c r="C49">
+        <v>707</v>
+      </c>
+      <c r="D49">
+        <v>69</v>
+      </c>
+      <c r="E49" s="4">
+        <f t="shared" si="4"/>
+        <v>229.8840579710145</v>
+      </c>
+      <c r="F49">
+        <v>363</v>
+      </c>
+      <c r="G49">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix board undo bug on gambits.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B256BE3C-9B2A-DA47-9723-11F6695D63BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C21A4928-24D2-1B43-9D17-BAE6E9AD4716}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -908,7 +908,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -2003,6 +2003,11 @@
         <v>71</v>
       </c>
     </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A50" s="6">
+        <v>46154</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Gambit better but still requires rerunGambits.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C21A4928-24D2-1B43-9D17-BAE6E9AD4716}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0751E77E-8213-FC4C-958C-532525F03F9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -1873,7 +1873,7 @@
         <v>69</v>
       </c>
       <c r="E44" s="4">
-        <f t="shared" ref="E44:E49" si="4">B44/D44</f>
+        <f t="shared" ref="E44:E50" si="4">B44/D44</f>
         <v>217.65217391304347</v>
       </c>
       <c r="F44">
@@ -2006,6 +2006,25 @@
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" s="6">
         <v>46154</v>
+      </c>
+      <c r="B50" s="9">
+        <v>15858</v>
+      </c>
+      <c r="C50">
+        <v>715</v>
+      </c>
+      <c r="D50">
+        <v>69</v>
+      </c>
+      <c r="E50" s="4">
+        <f t="shared" si="4"/>
+        <v>229.82608695652175</v>
+      </c>
+      <c r="F50">
+        <v>357</v>
+      </c>
+      <c r="G50">
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Gambit next plane feature.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ED5D7C7-0FA3-B14B-8317-D5A78085C3F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{439B792B-0CE1-654E-81A5-4AAFDCB0D4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -2056,23 +2056,23 @@
         <v>46156</v>
       </c>
       <c r="B52" s="9">
-        <v>15784</v>
+        <v>15896</v>
       </c>
       <c r="C52">
-        <v>692</v>
+        <v>696</v>
       </c>
       <c r="D52">
         <v>69</v>
       </c>
       <c r="E52" s="4">
         <f t="shared" si="4"/>
-        <v>228.75362318840581</v>
+        <v>230.37681159420291</v>
       </c>
       <c r="F52">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="G52">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Trays: show/hide, colors, json driven, board size.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5889565-AA09-8C47-9D8C-F9F228056B52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37A324C6-DA41-C443-9E2F-B313BD135808}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -1873,7 +1873,7 @@
         <v>69</v>
       </c>
       <c r="E44" s="4">
-        <f t="shared" ref="E44:E54" si="4">B44/D44</f>
+        <f t="shared" ref="E44:E55" si="4">B44/D44</f>
         <v>217.65217391304347</v>
       </c>
       <c r="F44">
@@ -2126,6 +2126,25 @@
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" s="6">
         <v>46159</v>
+      </c>
+      <c r="B55" s="9">
+        <v>16508</v>
+      </c>
+      <c r="C55">
+        <v>717</v>
+      </c>
+      <c r="D55">
+        <v>70</v>
+      </c>
+      <c r="E55" s="4">
+        <f t="shared" si="4"/>
+        <v>235.82857142857142</v>
+      </c>
+      <c r="F55">
+        <v>318</v>
+      </c>
+      <c r="G55">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Flesh out board and tray directories.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5043242A-81B0-DC43-A690-3FE0A1513481}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{446C8A42-D3E4-4C46-9DA1-4212CB144B3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -1873,7 +1873,7 @@
         <v>69</v>
       </c>
       <c r="E44" s="4">
-        <f t="shared" ref="E44:E56" si="4">B44/D44</f>
+        <f t="shared" ref="E44:E57" si="4">B44/D44</f>
         <v>217.65217391304347</v>
       </c>
       <c r="F44">
@@ -2174,6 +2174,25 @@
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57" s="6">
         <v>46161</v>
+      </c>
+      <c r="B57" s="9">
+        <v>17195</v>
+      </c>
+      <c r="C57">
+        <v>743</v>
+      </c>
+      <c r="D57">
+        <v>74</v>
+      </c>
+      <c r="E57" s="4">
+        <f t="shared" si="4"/>
+        <v>232.36486486486487</v>
+      </c>
+      <c r="F57">
+        <v>335</v>
+      </c>
+      <c r="G57">
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Piece render control flow.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{446C8A42-D3E4-4C46-9DA1-4212CB144B3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0FDF797-F9D6-C949-98E8-AE8878882899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -908,7 +908,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1873,7 +1873,7 @@
         <v>69</v>
       </c>
       <c r="E44" s="4">
-        <f t="shared" ref="E44:E57" si="4">B44/D44</f>
+        <f t="shared" ref="E44:E58" si="4">B44/D44</f>
         <v>217.65217391304347</v>
       </c>
       <c r="F44">
@@ -2193,6 +2193,30 @@
       </c>
       <c r="G57">
         <v>77</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A58" s="6">
+        <v>46162</v>
+      </c>
+      <c r="B58" s="9">
+        <v>17395</v>
+      </c>
+      <c r="C58">
+        <v>762</v>
+      </c>
+      <c r="D58">
+        <v>74</v>
+      </c>
+      <c r="E58" s="4">
+        <f t="shared" si="4"/>
+        <v>235.06756756756758</v>
+      </c>
+      <c r="F58">
+        <v>344</v>
+      </c>
+      <c r="G58">
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Debug vertical aspect error during piece expansion.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0FDF797-F9D6-C949-98E8-AE8878882899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBD84BC8-9B55-BC41-BF26-D579FF967585}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -908,7 +908,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -1873,7 +1873,7 @@
         <v>69</v>
       </c>
       <c r="E44" s="4">
-        <f t="shared" ref="E44:E58" si="4">B44/D44</f>
+        <f t="shared" ref="E44:E59" si="4">B44/D44</f>
         <v>217.65217391304347</v>
       </c>
       <c r="F44">
@@ -2217,6 +2217,30 @@
       </c>
       <c r="G58">
         <v>92</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A59" s="6">
+        <v>46163</v>
+      </c>
+      <c r="B59" s="9">
+        <v>17639</v>
+      </c>
+      <c r="C59">
+        <v>778</v>
+      </c>
+      <c r="D59">
+        <v>74</v>
+      </c>
+      <c r="E59" s="4">
+        <f t="shared" si="4"/>
+        <v>238.36486486486487</v>
+      </c>
+      <c r="F59">
+        <v>342</v>
+      </c>
+      <c r="G59">
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UI planel grouping via color.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBD84BC8-9B55-BC41-BF26-D579FF967585}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51BEFC61-8114-FE4A-8FF4-799BF6E72AFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -2224,23 +2224,23 @@
         <v>46163</v>
       </c>
       <c r="B59" s="9">
-        <v>17639</v>
+        <v>17779</v>
       </c>
       <c r="C59">
-        <v>778</v>
+        <v>781</v>
       </c>
       <c r="D59">
         <v>74</v>
       </c>
       <c r="E59" s="4">
         <f t="shared" si="4"/>
-        <v>238.36486486486487</v>
+        <v>240.25675675675674</v>
       </c>
       <c r="F59">
         <v>342</v>
       </c>
       <c r="G59">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Standardize control layer code.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51BEFC61-8114-FE4A-8FF4-799BF6E72AFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D994B078-EAB0-A444-87D6-439ACE1A7EE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -908,7 +908,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -2243,6 +2243,11 @@
         <v>98</v>
       </c>
     </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A60" s="6">
+        <v>46164</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Get level sep to work for trays.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D994B078-EAB0-A444-87D6-439ACE1A7EE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2406D781-9617-C54A-9543-7D2C228066C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="16940" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -1873,7 +1873,7 @@
         <v>69</v>
       </c>
       <c r="E44" s="4">
-        <f t="shared" ref="E44:E59" si="4">B44/D44</f>
+        <f t="shared" ref="E44:E60" si="4">B44/D44</f>
         <v>217.65217391304347</v>
       </c>
       <c r="F44">
@@ -2246,6 +2246,25 @@
     <row r="60" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A60" s="6">
         <v>46164</v>
+      </c>
+      <c r="B60" s="9">
+        <v>18042</v>
+      </c>
+      <c r="C60">
+        <v>785</v>
+      </c>
+      <c r="D60">
+        <v>74</v>
+      </c>
+      <c r="E60" s="4">
+        <f t="shared" si="4"/>
+        <v>243.81081081081081</v>
+      </c>
+      <c r="F60">
+        <v>343</v>
+      </c>
+      <c r="G60">
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Replace rest of Act 2 comics.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{542A2F3D-35B7-2C48-83E6-4D8277B98F4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{884AA5A1-4EE7-FB45-B502-CA1AD20D4AE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -908,7 +908,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -2463,6 +2463,30 @@
       <c r="A69" s="6">
         <v>46173</v>
       </c>
+      <c r="B69" s="9">
+        <v>17752</v>
+      </c>
+      <c r="C69">
+        <v>777</v>
+      </c>
+      <c r="D69">
+        <v>74</v>
+      </c>
+      <c r="E69" s="4">
+        <f t="shared" ref="E69" si="7">B69/D69</f>
+        <v>239.8918918918919</v>
+      </c>
+      <c r="F69">
+        <v>340</v>
+      </c>
+      <c r="G69">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A70" s="6">
+        <v>46174</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Tray default state is visible.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83F43CF6-BDA4-2146-8AE0-AFCA697CC40C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91D53557-F009-9245-A3E3-95126ADEE32E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -908,7 +908,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -2531,6 +2531,11 @@
         <v>95</v>
       </c>
     </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A72" s="6">
+        <v>46176</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update clues and quick start.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91D53557-F009-9245-A3E3-95126ADEE32E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9009D8BB-9608-6C4D-AECC-67F9F004E09C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -2473,7 +2473,7 @@
         <v>74</v>
       </c>
       <c r="E69" s="4">
-        <f t="shared" ref="E69:E71" si="7">B69/D69</f>
+        <f t="shared" ref="E69:E72" si="7">B69/D69</f>
         <v>239.8918918918919</v>
       </c>
       <c r="F69">
@@ -2534,6 +2534,25 @@
     <row r="72" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A72" s="6">
         <v>46176</v>
+      </c>
+      <c r="B72" s="9">
+        <v>18075</v>
+      </c>
+      <c r="C72">
+        <v>784</v>
+      </c>
+      <c r="D72">
+        <v>74</v>
+      </c>
+      <c r="E72" s="4">
+        <f t="shared" si="7"/>
+        <v>244.25675675675674</v>
+      </c>
+      <c r="F72">
+        <v>345</v>
+      </c>
+      <c r="G72">
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Create selections module, migrate tile listener.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9009D8BB-9608-6C4D-AECC-67F9F004E09C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13E97240-F261-9340-A67B-9141EC62F208}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -908,7 +908,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G72"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -2473,7 +2473,7 @@
         <v>74</v>
       </c>
       <c r="E69" s="4">
-        <f t="shared" ref="E69:E72" si="7">B69/D69</f>
+        <f t="shared" ref="E69:E73" si="7">B69/D69</f>
         <v>239.8918918918919</v>
       </c>
       <c r="F69">
@@ -2552,6 +2552,30 @@
         <v>345</v>
       </c>
       <c r="G72">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A73" s="6">
+        <v>46177</v>
+      </c>
+      <c r="B73" s="9">
+        <v>18268</v>
+      </c>
+      <c r="C73">
+        <v>797</v>
+      </c>
+      <c r="D73">
+        <v>77</v>
+      </c>
+      <c r="E73" s="4">
+        <f t="shared" si="7"/>
+        <v>237.24675324675326</v>
+      </c>
+      <c r="F73">
+        <v>351</v>
+      </c>
+      <c r="G73">
         <v>90</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Move pieces from tray to board.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13E97240-F261-9340-A67B-9141EC62F208}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC19E2E4-B634-9A4D-AB93-E21601DD20B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -908,7 +908,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G73"/>
+  <dimension ref="A1:G74"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -2579,6 +2579,11 @@
         <v>90</v>
       </c>
     </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A74" s="6">
+        <v>46178</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Setup uses selections, pass 1.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7FC226E-C9B6-764E-89FD-24F02FE1E1CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{769EEE9A-8FB0-6B4A-9638-1C18FCD4DA12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -2584,20 +2584,20 @@
         <v>46178</v>
       </c>
       <c r="B74" s="9">
-        <v>18483</v>
+        <v>18590</v>
       </c>
       <c r="C74">
-        <v>802</v>
+        <v>808</v>
       </c>
       <c r="D74">
         <v>77</v>
       </c>
       <c r="E74" s="4">
         <f t="shared" si="7"/>
-        <v>240.03896103896105</v>
+        <v>241.42857142857142</v>
       </c>
       <c r="F74">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="G74">
         <v>90</v>

</xml_diff>

<commit_message>
Setup uses selections pass 2.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{769EEE9A-8FB0-6B4A-9638-1C18FCD4DA12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F496C98-84C3-7A45-A3FA-242C9A8127B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -908,7 +908,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G74"/>
+  <dimension ref="A1:G75"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -2603,6 +2603,11 @@
         <v>90</v>
       </c>
     </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A75" s="6">
+        <v>46179</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Setup uses selections pass 3.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F496C98-84C3-7A45-A3FA-242C9A8127B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2A49BBC-4D23-644A-88C8-2160EA8C72E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -2473,7 +2473,7 @@
         <v>74</v>
       </c>
       <c r="E69" s="4">
-        <f t="shared" ref="E69:E74" si="7">B69/D69</f>
+        <f t="shared" ref="E69:E75" si="7">B69/D69</f>
         <v>239.8918918918919</v>
       </c>
       <c r="F69">
@@ -2606,6 +2606,25 @@
     <row r="75" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A75" s="6">
         <v>46179</v>
+      </c>
+      <c r="B75" s="9">
+        <v>18702</v>
+      </c>
+      <c r="C75">
+        <v>818</v>
+      </c>
+      <c r="D75">
+        <v>77</v>
+      </c>
+      <c r="E75" s="4">
+        <f t="shared" si="7"/>
+        <v>242.88311688311688</v>
+      </c>
+      <c r="F75">
+        <v>363</v>
+      </c>
+      <c r="G75">
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Improved initial placement of pieces in the trays, all three boards.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2A49BBC-4D23-644A-88C8-2160EA8C72E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA415567-CC73-AB42-BC6B-F05D37C269D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="30">
   <si>
     <t>Date</t>
   </si>
@@ -127,10 +127,24 @@
 grep -RIn "Seampoint: more imports" ./assets/3dc | wc
 grep -RIn "Seampoint: more global" ./assets/3dc | wc
 grep -RIn "Seampoint: more handlers" ./assets/3dc | wc
-grep -RIn "Seampoint: more handlers" ./assets/3dc | wc
 grep -RIn "Seampoint: more local" ./assets/3dc | wc
 grep -RIn "Seampoint: more tests" ./assets/3dc | wc
 grep -RIn "Seampoint: more " ./assets/3dc | wc</t>
+  </si>
+  <si>
+    <t>grep -R "Seampoint:" ./assets/3dc | wc</t>
+  </si>
+  <si>
+    <t>find ./assets/3dc -type d | wc</t>
+  </si>
+  <si>
+    <t>grep -RIn "export function" ./assets/3dc | wc</t>
+  </si>
+  <si>
+    <t>grep -R "Seampoint:" ./assets/3dc | wc -l
+grep -R "DEPRECATED" ./assets/3dc | wc -l
+grep -R "FIXME:" ./assets/3dc | wc -l
+find ./assets/3dc -type d | wc -l</t>
   </si>
 </sst>
 </file>
@@ -816,7 +830,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E93254FF-0763-D74B-A96C-EFEF852F1421}">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="54.1640625" customWidth="1"/>
@@ -896,9 +910,29 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="136" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2" ht="119" x14ac:dyDescent="0.2">
       <c r="B16" s="7" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B18" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B19" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B20" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" spans="2:2" ht="68" x14ac:dyDescent="0.2">
+      <c r="B22" s="7" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -908,7 +942,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G75"/>
+  <dimension ref="A1:G76"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -2473,7 +2507,7 @@
         <v>74</v>
       </c>
       <c r="E69" s="4">
-        <f t="shared" ref="E69:E75" si="7">B69/D69</f>
+        <f t="shared" ref="E69:E76" si="7">B69/D69</f>
         <v>239.8918918918919</v>
       </c>
       <c r="F69">
@@ -2625,6 +2659,30 @@
       </c>
       <c r="G75">
         <v>89</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A76" s="6">
+        <v>46180</v>
+      </c>
+      <c r="B76" s="9">
+        <v>19153</v>
+      </c>
+      <c r="C76">
+        <v>824</v>
+      </c>
+      <c r="D76">
+        <v>77</v>
+      </c>
+      <c r="E76" s="4">
+        <f t="shared" si="7"/>
+        <v>248.74025974025975</v>
+      </c>
+      <c r="F76">
+        <v>366</v>
+      </c>
+      <c r="G76">
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Setup undo phase 1.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C1575A2-AA16-0C40-A847-A9AFD4A4B7EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77A331B1-D444-2E45-ADCE-7C5DB2CA5CFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -2507,7 +2507,7 @@
         <v>74</v>
       </c>
       <c r="E69" s="4">
-        <f t="shared" ref="E69:E77" si="7">B69/D69</f>
+        <f t="shared" ref="E69:E78" si="7">B69/D69</f>
         <v>239.8918918918919</v>
       </c>
       <c r="F69">
@@ -2712,6 +2712,25 @@
     <row r="78" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A78" s="6">
         <v>46182</v>
+      </c>
+      <c r="B78" s="9">
+        <v>19505</v>
+      </c>
+      <c r="C78">
+        <v>856</v>
+      </c>
+      <c r="D78">
+        <v>79</v>
+      </c>
+      <c r="E78" s="4">
+        <f t="shared" si="7"/>
+        <v>246.8987341772152</v>
+      </c>
+      <c r="F78">
+        <v>382</v>
+      </c>
+      <c r="G78">
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Panel logic for setup makeBoard; tiles, trays, pieces still to do.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2923DCAE-1DED-2D4D-8470-20BD703082A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34B73FA2-3AC4-4C4E-8866-1AFE583018F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -942,7 +942,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G80"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -2507,7 +2507,7 @@
         <v>74</v>
       </c>
       <c r="E69" s="4">
-        <f t="shared" ref="E69:E80" si="7">B69/D69</f>
+        <f t="shared" ref="E69:E81" si="7">B69/D69</f>
         <v>239.8918918918919</v>
       </c>
       <c r="F69">
@@ -2779,6 +2779,30 @@
       </c>
       <c r="G80">
         <v>95</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A81" s="6">
+        <v>46185</v>
+      </c>
+      <c r="B81" s="9">
+        <v>19735</v>
+      </c>
+      <c r="C81">
+        <v>872</v>
+      </c>
+      <c r="D81">
+        <v>79</v>
+      </c>
+      <c r="E81" s="4">
+        <f t="shared" si="7"/>
+        <v>249.81012658227849</v>
+      </c>
+      <c r="F81">
+        <v>401</v>
+      </c>
+      <c r="G81">
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update clues & dates.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{466B3789-A148-274C-A511-50BF2F167A28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EEABA18-842E-1F47-A5A1-CAA37C702AFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -2834,23 +2834,23 @@
         <v>46187</v>
       </c>
       <c r="B83" s="9">
-        <v>18927</v>
+        <v>18922</v>
       </c>
       <c r="C83">
-        <v>876</v>
+        <v>874</v>
       </c>
       <c r="D83">
         <v>79</v>
       </c>
       <c r="E83" s="4">
         <f t="shared" si="7"/>
-        <v>239.58227848101265</v>
+        <v>239.51898734177215</v>
       </c>
       <c r="F83">
         <v>406</v>
       </c>
       <c r="G83">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
1st level move button restraints.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2622DD53-8503-164E-84D6-E62ACE4EDEFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33D2C440-251E-E84E-A4B3-10F20AB1048D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -2507,7 +2507,7 @@
         <v>74</v>
       </c>
       <c r="E69" s="4">
-        <f t="shared" ref="E69:E83" si="7">B69/D69</f>
+        <f t="shared" ref="E69:E84" si="7">B69/D69</f>
         <v>239.8918918918919</v>
       </c>
       <c r="F69">
@@ -2856,6 +2856,25 @@
     <row r="84" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A84" s="6">
         <v>46188</v>
+      </c>
+      <c r="B84" s="9">
+        <v>19192</v>
+      </c>
+      <c r="C84">
+        <v>881</v>
+      </c>
+      <c r="D84">
+        <v>79</v>
+      </c>
+      <c r="E84" s="4">
+        <f t="shared" si="7"/>
+        <v>242.9367088607595</v>
+      </c>
+      <c r="F84">
+        <v>407</v>
+      </c>
+      <c r="G84">
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add two stack move buttons.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33D2C440-251E-E84E-A4B3-10F20AB1048D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CE01294-E322-1C49-B6C3-5CD72139AC8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -942,7 +942,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G84"/>
+  <dimension ref="A1:G85"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -2877,6 +2877,11 @@
         <v>83</v>
       </c>
     </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A85" s="6">
+        <v>46189</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Move pieces around the board.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFA7899A-E3CD-0647-9720-97390AD3A58D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A43EFC51-F902-F74A-803E-2B981D590E8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -2882,20 +2882,20 @@
         <v>46189</v>
       </c>
       <c r="B85" s="9">
-        <v>19355</v>
+        <v>19487</v>
       </c>
       <c r="C85">
-        <v>887</v>
+        <v>892</v>
       </c>
       <c r="D85">
         <v>79</v>
       </c>
       <c r="E85" s="4">
         <f t="shared" si="7"/>
-        <v>245</v>
+        <v>246.67088607594937</v>
       </c>
       <c r="F85">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="G85">
         <v>85</v>

</xml_diff>

<commit_message>
Plumbing for undo moves.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A43EFC51-F902-F74A-803E-2B981D590E8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBCFB55A-81C1-684C-AB2B-AC0B0FADE737}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -942,7 +942,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G85"/>
+  <dimension ref="A1:G86"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -2507,7 +2507,7 @@
         <v>74</v>
       </c>
       <c r="E69" s="4">
-        <f t="shared" ref="E69:E85" si="7">B69/D69</f>
+        <f t="shared" ref="E69:E86" si="7">B69/D69</f>
         <v>239.8918918918919</v>
       </c>
       <c r="F69">
@@ -2899,6 +2899,30 @@
       </c>
       <c r="G85">
         <v>85</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A86" s="6">
+        <v>46190</v>
+      </c>
+      <c r="B86" s="9">
+        <v>19689</v>
+      </c>
+      <c r="C86">
+        <v>896</v>
+      </c>
+      <c r="D86">
+        <v>79</v>
+      </c>
+      <c r="E86" s="4">
+        <f t="shared" si="7"/>
+        <v>249.22784810126583</v>
+      </c>
+      <c r="F86">
+        <v>411</v>
+      </c>
+      <c r="G86">
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Push & Pop panel lines.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6185543B-8743-524F-9815-7C5625BD434E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2CF6D6F-1570-9643-945B-2E910FB6E05E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -2906,23 +2906,23 @@
         <v>46190</v>
       </c>
       <c r="B86" s="9">
-        <v>19689</v>
+        <v>19538</v>
       </c>
       <c r="C86">
-        <v>896</v>
+        <v>881</v>
       </c>
       <c r="D86">
         <v>79</v>
       </c>
       <c r="E86" s="4">
         <f t="shared" si="7"/>
-        <v>249.22784810126583</v>
+        <v>247.31645569620252</v>
       </c>
       <c r="F86">
-        <v>411</v>
+        <v>406</v>
       </c>
       <c r="G86">
-        <v>106</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Undo/redo/RW/FF/load/save for quadrant gambits.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49BA9CA8-EDE1-EB40-BF40-EFAAD63ABA37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F26661D-ADC7-1148-9A63-6355F7857F8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -2507,7 +2507,7 @@
         <v>74</v>
       </c>
       <c r="E69" s="4">
-        <f t="shared" ref="E69:E86" si="7">B69/D69</f>
+        <f t="shared" ref="E69:E87" si="7">B69/D69</f>
         <v>239.8918918918919</v>
       </c>
       <c r="F69">
@@ -2928,6 +2928,25 @@
     <row r="87" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A87" s="6">
         <v>46191</v>
+      </c>
+      <c r="B87" s="9">
+        <v>19738</v>
+      </c>
+      <c r="C87">
+        <v>896</v>
+      </c>
+      <c r="D87">
+        <v>79</v>
+      </c>
+      <c r="E87" s="4">
+        <f t="shared" si="7"/>
+        <v>249.84810126582278</v>
+      </c>
+      <c r="F87">
+        <v>416</v>
+      </c>
+      <c r="G87">
+        <v>102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deadcode & todo updates.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F26661D-ADC7-1148-9A63-6355F7857F8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{436ECC39-B60A-474E-9BAF-6F05D08D268D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -942,7 +942,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G87"/>
+  <dimension ref="A1:G88"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -2949,6 +2949,11 @@
         <v>102</v>
       </c>
     </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A88" s="6">
+        <v>46192</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Cross panel button affordances.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56D3E05F-66E1-4641-8CED-BEB34376B3D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C518E7C3-AB6C-8349-A0CF-A3EBB305F339}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -942,7 +942,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G88"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -2973,6 +2973,11 @@
         <v>98</v>
       </c>
     </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A89" s="6">
+        <v>46193</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Fixed White/Black radio buttons in move panel.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D97F8D7-0DEC-694B-B08D-45E0080D4960}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F185DE5A-F46A-A349-923E-9A90D5FFAADA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
+    <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="2" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
   <sheets>
     <sheet name="Docs" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="32">
   <si>
     <t>Date</t>
   </si>
@@ -145,6 +145,12 @@
 grep -R "DEPRECATED" ./assets/3dc | wc -l
 grep -R "FIXME:" ./assets/3dc | wc -l
 find ./assets/3dc -type d | wc -l</t>
+  </si>
+  <si>
+    <t>wc -l $(find ./assets/3dc -type f) | sort -n</t>
+  </si>
+  <si>
+    <t>find ./assets/3dc -type f ! -name ".DS_Store" -exec wc -l {} + | sort -nr</t>
   </si>
 </sst>
 </file>
@@ -830,7 +836,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E93254FF-0763-D74B-A96C-EFEF852F1421}">
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="54.1640625" customWidth="1"/>
@@ -933,6 +939,16 @@
     <row r="22" spans="2:2" ht="68" x14ac:dyDescent="0.2">
       <c r="B22" s="7" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B24" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="25" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B25" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Normalize move entry and payload/selections order.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F185DE5A-F46A-A349-923E-9A90D5FFAADA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0FBC5F0-3E17-D64A-BEAB-0FDAD4C260F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="2" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
+    <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
   <sheets>
     <sheet name="Docs" sheetId="2" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Commands" sheetId="3" r:id="rId3"/>
     <sheet name="3DC" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -30,7 +30,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -116,13 +115,6 @@
     <t>TODOs</t>
   </si>
   <si>
-    <t>wc -l $(find ./assets/3dc -type f);
-grep -RIn "function" ./assets/3dc | wc;
-find ./assets/3dc -type f -name "*.js" | wc;
-grep -RIn "export function" ./assets/3dc | wc
-grep -RIn "TODO:" ./assets/3dc | wc</t>
-  </si>
-  <si>
     <t>grep -RIn "Seampoint: more objects" ./assets/3dc | wc
 grep -RIn "Seampoint: more imports" ./assets/3dc | wc
 grep -RIn "Seampoint: more global" ./assets/3dc | wc
@@ -151,6 +143,13 @@
   </si>
   <si>
     <t>find ./assets/3dc -type f ! -name ".DS_Store" -exec wc -l {} + | sort -nr</t>
+  </si>
+  <si>
+    <t>find ./assets/3dc -type f ! -name ".DS_Store" -exec wc -l {} + | sort -n;
+grep -RIn "function" ./assets/3dc | wc;
+find ./assets/3dc -type f -name "*.js" | wc;
+grep -RIn "export function" ./assets/3dc | wc
+grep -RIn "TODO:" ./assets/3dc | wc</t>
   </si>
 </sst>
 </file>
@@ -911,44 +910,44 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="85" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" ht="102" x14ac:dyDescent="0.2">
       <c r="B14" s="7" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="119" x14ac:dyDescent="0.2">
       <c r="B16" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22" spans="2:2" ht="68" x14ac:dyDescent="0.2">
       <c r="B22" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="24" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -958,7 +957,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G90"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -2523,7 +2522,7 @@
         <v>74</v>
       </c>
       <c r="E69" s="4">
-        <f t="shared" ref="E69:E89" si="7">B69/D69</f>
+        <f t="shared" ref="E69:E90" si="7">B69/D69</f>
         <v>239.8918918918919</v>
       </c>
       <c r="F69">
@@ -3011,6 +3010,30 @@
       </c>
       <c r="G89">
         <v>96</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A90" s="6">
+        <v>46194</v>
+      </c>
+      <c r="B90" s="9">
+        <v>19718</v>
+      </c>
+      <c r="C90">
+        <v>908</v>
+      </c>
+      <c r="D90">
+        <v>79</v>
+      </c>
+      <c r="E90" s="4">
+        <f t="shared" si="7"/>
+        <v>249.59493670886076</v>
+      </c>
+      <c r="F90">
+        <v>423</v>
+      </c>
+      <c r="G90">
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Promotion sans queen mesh.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{546BF2A6-425D-A846-8F26-FDE85DA93B62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD116760-6D4A-9449-8E4D-36349CF799AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -2522,7 +2522,7 @@
         <v>74</v>
       </c>
       <c r="E69" s="4">
-        <f t="shared" ref="E69:E90" si="7">B69/D69</f>
+        <f t="shared" ref="E69:E91" si="7">B69/D69</f>
         <v>239.8918918918919</v>
       </c>
       <c r="F69">
@@ -3039,6 +3039,25 @@
     <row r="91" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A91" s="6">
         <v>46195</v>
+      </c>
+      <c r="B91" s="9">
+        <v>19952</v>
+      </c>
+      <c r="C91">
+        <v>927</v>
+      </c>
+      <c r="D91">
+        <v>79</v>
+      </c>
+      <c r="E91" s="4">
+        <f t="shared" si="7"/>
+        <v>252.55696202531647</v>
+      </c>
+      <c r="F91">
+        <v>429</v>
+      </c>
+      <c r="G91">
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Stem out move makeEntries and assembleLines.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD116760-6D4A-9449-8E4D-36349CF799AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{180D9582-7FC6-2D40-9992-A8849204DF61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -3041,23 +3041,23 @@
         <v>46195</v>
       </c>
       <c r="B91" s="9">
-        <v>19952</v>
+        <v>20146</v>
       </c>
       <c r="C91">
-        <v>927</v>
+        <v>934</v>
       </c>
       <c r="D91">
         <v>79</v>
       </c>
       <c r="E91" s="4">
         <f t="shared" si="7"/>
-        <v>252.55696202531647</v>
+        <v>255.01265822784811</v>
       </c>
       <c r="F91">
-        <v>429</v>
+        <v>433</v>
       </c>
       <c r="G91">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
New approach; pieceList and trays only - POC.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{180D9582-7FC6-2D40-9992-A8849204DF61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCEC2633-8C7B-C348-BB4A-03D88C61EF86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -957,7 +957,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G91"/>
+  <dimension ref="A1:G92"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -2522,7 +2522,7 @@
         <v>74</v>
       </c>
       <c r="E69" s="4">
-        <f t="shared" ref="E69:E91" si="7">B69/D69</f>
+        <f t="shared" ref="E69:E92" si="7">B69/D69</f>
         <v>239.8918918918919</v>
       </c>
       <c r="F69">
@@ -3058,6 +3058,30 @@
       </c>
       <c r="G91">
         <v>92</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A92" s="6">
+        <v>46196</v>
+      </c>
+      <c r="B92" s="9">
+        <v>20465</v>
+      </c>
+      <c r="C92">
+        <v>950</v>
+      </c>
+      <c r="D92">
+        <v>79</v>
+      </c>
+      <c r="E92" s="4">
+        <f t="shared" si="7"/>
+        <v>259.05063291139243</v>
+      </c>
+      <c r="F92">
+        <v>445</v>
+      </c>
+      <c r="G92">
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rest of base moves.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{543DE055-0CED-6E42-918A-833AD2D50477}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E0C2082-0828-FC40-A150-CC08BAF3E335}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -957,7 +957,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G93"/>
+  <dimension ref="A1:G94"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -3108,6 +3108,11 @@
         <v>83</v>
       </c>
     </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A94" s="6">
+        <v>46198</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Rest of non fission captures.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E0C2082-0828-FC40-A150-CC08BAF3E335}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CB389C6-3F03-BA4E-B92E-4C35C940894C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -2522,7 +2522,7 @@
         <v>74</v>
       </c>
       <c r="E69" s="4">
-        <f t="shared" ref="E69:E93" si="7">B69/D69</f>
+        <f t="shared" ref="E69:E94" si="7">B69/D69</f>
         <v>239.8918918918919</v>
       </c>
       <c r="F69">
@@ -3111,6 +3111,25 @@
     <row r="94" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A94" s="6">
         <v>46198</v>
+      </c>
+      <c r="B94" s="9">
+        <v>20723</v>
+      </c>
+      <c r="C94">
+        <v>933</v>
+      </c>
+      <c r="D94">
+        <v>79</v>
+      </c>
+      <c r="E94" s="4">
+        <f t="shared" si="7"/>
+        <v>262.31645569620252</v>
+      </c>
+      <c r="F94">
+        <v>432</v>
+      </c>
+      <c r="G94">
+        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fission, 16 permutations, just eligibility.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CB389C6-3F03-BA4E-B92E-4C35C940894C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7754BEA5-40DB-C64A-A09B-289145FE84DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -957,7 +957,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G94"/>
+  <dimension ref="A1:G95"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -2522,7 +2522,7 @@
         <v>74</v>
       </c>
       <c r="E69" s="4">
-        <f t="shared" ref="E69:E94" si="7">B69/D69</f>
+        <f t="shared" ref="E69:E95" si="7">B69/D69</f>
         <v>239.8918918918919</v>
       </c>
       <c r="F69">
@@ -3130,6 +3130,30 @@
       </c>
       <c r="G94">
         <v>81</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A95" s="6">
+        <v>46199</v>
+      </c>
+      <c r="B95" s="9">
+        <v>20928</v>
+      </c>
+      <c r="C95">
+        <v>936</v>
+      </c>
+      <c r="D95">
+        <v>79</v>
+      </c>
+      <c r="E95" s="4">
+        <f t="shared" si="7"/>
+        <v>264.91139240506328</v>
+      </c>
+      <c r="F95">
+        <v>432</v>
+      </c>
+      <c r="G95">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fission moves (4): entries, lines, and pieces.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7754BEA5-40DB-C64A-A09B-289145FE84DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C7FD67B-727E-1746-8CBC-B3F5F8369A0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -957,7 +957,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G95"/>
+  <dimension ref="A1:G96"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -3156,6 +3156,11 @@
         <v>82</v>
       </c>
     </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A96" s="6">
+        <v>46200</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
8/16 fissions, but B/D click order problematic.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C7FD67B-727E-1746-8CBC-B3F5F8369A0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{450D5125-8DCB-FC44-80C6-DD47458F44E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -838,7 +838,7 @@
   <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="54.1640625" customWidth="1"/>
+    <col min="2" max="2" width="55.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -2522,7 +2522,7 @@
         <v>74</v>
       </c>
       <c r="E69" s="4">
-        <f t="shared" ref="E69:E95" si="7">B69/D69</f>
+        <f t="shared" ref="E69:E96" si="7">B69/D69</f>
         <v>239.8918918918919</v>
       </c>
       <c r="F69">
@@ -3159,6 +3159,25 @@
     <row r="96" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A96" s="6">
         <v>46200</v>
+      </c>
+      <c r="B96" s="9">
+        <v>21558</v>
+      </c>
+      <c r="C96">
+        <v>939</v>
+      </c>
+      <c r="D96">
+        <v>79</v>
+      </c>
+      <c r="E96" s="4">
+        <f t="shared" si="7"/>
+        <v>272.88607594936707</v>
+      </c>
+      <c r="F96">
+        <v>435</v>
+      </c>
+      <c r="G96">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correct click order for fission moves.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{450D5125-8DCB-FC44-80C6-DD47458F44E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E31B7B8-73EC-564A-A663-4DF508755BFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -957,7 +957,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G96"/>
+  <dimension ref="A1:G97"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -3180,6 +3180,11 @@
         <v>82</v>
       </c>
     </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A97" s="6">
+        <v>46201</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Raise and lower duke (all but bishop leaves).
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E31B7B8-73EC-564A-A663-4DF508755BFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27CD274B-0611-4F44-B4D8-8CFEFBAFFB03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -2522,7 +2522,7 @@
         <v>74</v>
       </c>
       <c r="E69" s="4">
-        <f t="shared" ref="E69:E96" si="7">B69/D69</f>
+        <f t="shared" ref="E69:E97" si="7">B69/D69</f>
         <v>239.8918918918919</v>
       </c>
       <c r="F69">
@@ -3180,9 +3180,28 @@
         <v>82</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A97" s="6">
         <v>46201</v>
+      </c>
+      <c r="B97" s="9">
+        <v>21791</v>
+      </c>
+      <c r="C97">
+        <v>939</v>
+      </c>
+      <c r="D97">
+        <v>79</v>
+      </c>
+      <c r="E97" s="4">
+        <f t="shared" si="7"/>
+        <v>275.8354430379747</v>
+      </c>
+      <c r="F97">
+        <v>435</v>
+      </c>
+      <c r="G97">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finish en passant and castling.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27CD274B-0611-4F44-B4D8-8CFEFBAFFB03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D52D31D5-29DD-4D4D-8186-FF682ADF562F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="Commands" sheetId="3" r:id="rId3"/>
     <sheet name="3DC" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -30,6 +30,7 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -957,7 +958,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G97"/>
+  <dimension ref="A1:G98"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -3204,6 +3205,11 @@
         <v>82</v>
       </c>
     </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A98" s="6">
+        <v>46202</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Finish setup affordances execpt for stack.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8212FF45-354A-B54A-B466-85C1CCBD1974}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FDD7FC0-38BE-F74E-A060-4E8971172A1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-20800" windowWidth="25660" windowHeight="18780" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -2523,7 +2523,7 @@
         <v>74</v>
       </c>
       <c r="E69" s="4">
-        <f t="shared" ref="E69:E98" si="7">B69/D69</f>
+        <f t="shared" ref="E69:E99" si="7">B69/D69</f>
         <v>239.8918918918919</v>
       </c>
       <c r="F69">
@@ -3232,6 +3232,25 @@
     <row r="99" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A99" s="6">
         <v>46203</v>
+      </c>
+      <c r="B99" s="9">
+        <v>22116</v>
+      </c>
+      <c r="C99">
+        <v>952</v>
+      </c>
+      <c r="D99">
+        <v>80</v>
+      </c>
+      <c r="E99" s="4">
+        <f t="shared" si="7"/>
+        <v>276.45</v>
+      </c>
+      <c r="F99">
+        <v>448</v>
+      </c>
+      <c r="G99">
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
QC applyEntry and advsqs.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E847E01D-D83B-CC4D-B161-59F94DDDC4F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{732102B2-D35F-CB40-B11A-F51D523E3A61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="19500" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -958,7 +958,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA36453E-C248-E840-8857-250AF6BAF4EC}">
-  <dimension ref="A1:G108"/>
+  <dimension ref="A1:G109"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -3469,6 +3469,11 @@
         <v>100</v>
       </c>
     </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A109" s="6">
+        <v>46213</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Debug advsqs removal after place or move.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{732102B2-D35F-CB40-B11A-F51D523E3A61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF07EFAE-5225-4B46-9BAB-E7C315E3CD96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="19500" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -2523,7 +2523,7 @@
         <v>74</v>
       </c>
       <c r="E69" s="4">
-        <f t="shared" ref="E69:E108" si="7">B69/D69</f>
+        <f t="shared" ref="E69:E109" si="7">B69/D69</f>
         <v>239.8918918918919</v>
       </c>
       <c r="F69">
@@ -3472,6 +3472,25 @@
     <row r="109" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A109" s="6">
         <v>46213</v>
+      </c>
+      <c r="B109" s="9">
+        <v>23987</v>
+      </c>
+      <c r="C109">
+        <v>978</v>
+      </c>
+      <c r="D109">
+        <v>80</v>
+      </c>
+      <c r="E109" s="4">
+        <f t="shared" si="7"/>
+        <v>299.83749999999998</v>
+      </c>
+      <c r="F109">
+        <v>464</v>
+      </c>
+      <c r="G109">
+        <v>103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Several critical visual tweaks.
</commit_message>
<xml_diff>
--- a/meta/project.xlsx
+++ b/meta/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3007FBB8-C079-CB48-A3EF-9B61BE8301D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE754CF4-8433-F848-B88F-26335E9DD179}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51140" yWindow="-21000" windowWidth="25660" windowHeight="19500" activeTab="3" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -3498,7 +3498,7 @@
         <v>46214</v>
       </c>
       <c r="B110" s="9">
-        <v>23991</v>
+        <v>23999</v>
       </c>
       <c r="C110">
         <v>978</v>
@@ -3508,7 +3508,7 @@
       </c>
       <c r="E110" s="4">
         <f t="shared" si="7"/>
-        <v>299.88749999999999</v>
+        <v>299.98750000000001</v>
       </c>
       <c r="F110">
         <v>464</v>

</xml_diff>